<commit_message>
feat: manager utility/rent billing status + web-compatible flows
- BuildingBillingScreen: dùng API thật, chỉ hóa đơn tiền nhà (RENT) theo BĐS
- BillingManagementScreen: hub chỉ tính RENT; fix Alert xác nhận trên web
- UtilityBillingScreen: đơn giá điện = tổng tiền EVN / tổng kWh; nhập tay chỉ số cũ/mới;
  panel trạng thái điện/nước theo nhà + tab Lịch sử lấy dữ liệu thật; format số tiền
- import panels: ẩn báo "hợp lệ" khi import lỗi (web Alert)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend-web/public/templates/SLMS2026_import_dot1_khoi_tao.xlsx
+++ b/frontend-web/public/templates/SLMS2026_import_dot1_khoi_tao.xlsx
@@ -631,13 +631,13 @@
         <v>NGUYEN_CAN</v>
       </c>
       <c r="D9" t="str">
-        <v>Không</v>
+        <v>Có</v>
       </c>
       <c r="E9" t="str">
         <v>Có</v>
       </c>
       <c r="F9" t="str">
-        <v>NGUYEN_CAN — không dòng cải tạo, chỉ mua TB</v>
+        <v>NGUYEN_CAN — 1 hạng mục cải tạo nhẹ + mua TB</v>
       </c>
     </row>
     <row r="10">
@@ -988,7 +988,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M16"/>
+  <dimension ref="A1:O16"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -1003,6 +1003,8 @@
     <col min="11" max="11" width="18.83203125" customWidth="1"/>
     <col min="12" max="12" width="18.83203125" customWidth="1"/>
     <col min="13" max="13" width="18.83203125" customWidth="1"/>
+    <col min="14" max="14" width="18.83203125" customWidth="1"/>
+    <col min="15" max="15" width="18.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1025,24 +1027,30 @@
         <v>Diện tích (m²)</v>
       </c>
       <c r="G1" t="str">
+        <v>Chiều dài (m)</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Chiều rộng (m)</v>
+      </c>
+      <c r="I1" t="str">
         <v>Tổng số tầng</v>
       </c>
-      <c r="H1" t="str">
+      <c r="J1" t="str">
         <v>Tổng số phòng</v>
       </c>
-      <c r="I1" t="str">
+      <c r="K1" t="str">
         <v>Tên chủ nhà</v>
       </c>
-      <c r="J1" t="str">
+      <c r="L1" t="str">
         <v>Tổng tiền thuê</v>
       </c>
-      <c r="K1" t="str">
+      <c r="M1" t="str">
         <v>Ngày bắt đầu</v>
       </c>
-      <c r="L1" t="str">
+      <c r="N1" t="str">
         <v>Ngày kết thúc</v>
       </c>
-      <c r="M1" t="str">
+      <c r="O1" t="str">
         <v>Mô tả chi tiết</v>
       </c>
     </row>
@@ -1066,24 +1074,30 @@
         <v>180</v>
       </c>
       <c r="G2">
+        <v>15.9</v>
+      </c>
+      <c r="H2">
+        <v>11.3</v>
+      </c>
+      <c r="I2">
         <v>2</v>
       </c>
-      <c r="H2">
+      <c r="J2">
         <v>5</v>
       </c>
-      <c r="I2" t="str">
+      <c r="K2" t="str">
         <v>Trần Minh Tuấn</v>
       </c>
-      <c r="J2">
+      <c r="L2">
         <v>450000000</v>
       </c>
-      <c r="K2" t="str">
+      <c r="M2" t="str">
         <v>2026-03-01</v>
       </c>
-      <c r="L2" t="str">
+      <c r="N2" t="str">
         <v>2029-02-28</v>
       </c>
-      <c r="M2" t="str">
+      <c r="O2" t="str">
         <v>Biệt thự thuê nguyên căn — chờ cải tạo đợt 2.</v>
       </c>
     </row>
@@ -1107,24 +1121,30 @@
         <v>95</v>
       </c>
       <c r="G3">
+        <v>11.5</v>
+      </c>
+      <c r="H3">
+        <v>8.3</v>
+      </c>
+      <c r="I3">
         <v>2</v>
       </c>
-      <c r="H3">
+      <c r="J3">
         <v>4</v>
       </c>
-      <c r="I3" t="str">
+      <c r="K3" t="str">
         <v>Phạm Văn Đức</v>
       </c>
-      <c r="J3">
+      <c r="L3">
         <v>280000000</v>
       </c>
-      <c r="K3" t="str">
+      <c r="M3" t="str">
         <v>2026-05-01</v>
       </c>
-      <c r="L3" t="str">
+      <c r="N3" t="str">
         <v>2031-04-30</v>
       </c>
-      <c r="M3" t="str">
+      <c r="O3" t="str">
         <v>Vào ở ngay — chỉ TB chủ bàn giao, không cải tạo.</v>
       </c>
     </row>
@@ -1148,24 +1168,30 @@
         <v>200</v>
       </c>
       <c r="G4">
+        <v>16.7</v>
+      </c>
+      <c r="H4">
+        <v>12</v>
+      </c>
+      <c r="I4">
         <v>1</v>
       </c>
-      <c r="H4">
+      <c r="J4">
         <v>4</v>
       </c>
-      <c r="I4" t="str">
+      <c r="K4" t="str">
         <v>Đặng Quốc Bảo</v>
       </c>
-      <c r="J4">
+      <c r="L4">
         <v>550000000</v>
       </c>
-      <c r="K4" t="str">
+      <c r="M4" t="str">
         <v>2026-09-01</v>
       </c>
-      <c r="L4" t="str">
+      <c r="N4" t="str">
         <v>2031-08-31</v>
       </c>
-      <c r="M4" t="str">
+      <c r="O4" t="str">
         <v>Cải tạo hoàn thiện, không mua TB mới.</v>
       </c>
     </row>
@@ -1189,24 +1215,30 @@
         <v>55</v>
       </c>
       <c r="G5">
+        <v>8.8</v>
+      </c>
+      <c r="H5">
+        <v>6.2</v>
+      </c>
+      <c r="I5">
         <v>1</v>
       </c>
-      <c r="H5">
+      <c r="J5">
         <v>1</v>
       </c>
-      <c r="I5" t="str">
+      <c r="K5" t="str">
         <v>Nguyễn Thu Hà</v>
       </c>
-      <c r="J5">
+      <c r="L5">
         <v>180000000</v>
       </c>
-      <c r="K5" t="str">
+      <c r="M5" t="str">
         <v>2026-06-01</v>
       </c>
-      <c r="L5" t="str">
+      <c r="N5" t="str">
         <v>2027-05-31</v>
       </c>
-      <c r="M5" t="str">
+      <c r="O5" t="str">
         <v>Nhà trống hoàn toàn, không cải tạo.</v>
       </c>
     </row>
@@ -1230,24 +1262,30 @@
         <v>120</v>
       </c>
       <c r="G6">
+        <v>13</v>
+      </c>
+      <c r="H6">
+        <v>9.2</v>
+      </c>
+      <c r="I6">
         <v>3</v>
       </c>
-      <c r="H6">
+      <c r="J6">
         <v>8</v>
       </c>
-      <c r="I6" t="str">
+      <c r="K6" t="str">
         <v>Lê Thị Hương</v>
       </c>
-      <c r="J6">
+      <c r="L6">
         <v>320000000</v>
       </c>
-      <c r="K6" t="str">
+      <c r="M6" t="str">
         <v>2026-04-01</v>
       </c>
-      <c r="L6" t="str">
+      <c r="N6" t="str">
         <v>2028-03-31</v>
       </c>
-      <c r="M6" t="str">
+      <c r="O6" t="str">
         <v>Thuê nguyên căn từ chủ — đợt 2 chia 5 phòng khai thác.</v>
       </c>
     </row>
@@ -1271,24 +1309,30 @@
         <v>160</v>
       </c>
       <c r="G7">
+        <v>15</v>
+      </c>
+      <c r="H7">
+        <v>10.7</v>
+      </c>
+      <c r="I7">
         <v>4</v>
       </c>
-      <c r="H7">
+      <c r="J7">
         <v>10</v>
       </c>
-      <c r="I7" t="str">
+      <c r="K7" t="str">
         <v>Võ Minh Khang</v>
       </c>
-      <c r="J7">
+      <c r="L7">
         <v>380000000</v>
       </c>
-      <c r="K7" t="str">
+      <c r="M7" t="str">
         <v>2026-02-01</v>
       </c>
-      <c r="L7" t="str">
+      <c r="N7" t="str">
         <v>2029-01-31</v>
       </c>
-      <c r="M7" t="str">
+      <c r="O7" t="str">
         <v>Nhà trọ lớn — chia 8 phòng khai thác.</v>
       </c>
     </row>
@@ -1312,24 +1356,30 @@
         <v>75</v>
       </c>
       <c r="G8">
+        <v>10.2</v>
+      </c>
+      <c r="H8">
+        <v>7.4</v>
+      </c>
+      <c r="I8">
         <v>2</v>
       </c>
-      <c r="H8">
+      <c r="J8">
         <v>3</v>
       </c>
-      <c r="I8" t="str">
+      <c r="K8" t="str">
         <v>Hoàng Thị Lan</v>
       </c>
-      <c r="J8">
+      <c r="L8">
         <v>220000000</v>
       </c>
-      <c r="K8" t="str">
+      <c r="M8" t="str">
         <v>2026-07-01</v>
       </c>
-      <c r="L8" t="str">
+      <c r="N8" t="str">
         <v>2028-06-30</v>
       </c>
-      <c r="M8" t="str">
+      <c r="O8" t="str">
         <v>Nhà nhỏ chia 3 phòng — không TB bàn giao.</v>
       </c>
     </row>
@@ -1353,25 +1403,31 @@
         <v>68</v>
       </c>
       <c r="G9">
+        <v>9.8</v>
+      </c>
+      <c r="H9">
+        <v>6.9</v>
+      </c>
+      <c r="I9">
         <v>1</v>
       </c>
-      <c r="H9">
+      <c r="J9">
         <v>2</v>
       </c>
-      <c r="I9" t="str">
+      <c r="K9" t="str">
         <v>Bùi Văn Nam</v>
       </c>
-      <c r="J9">
+      <c r="L9">
         <v>195000000</v>
       </c>
-      <c r="K9" t="str">
+      <c r="M9" t="str">
         <v>2026-08-01</v>
       </c>
-      <c r="L9" t="str">
+      <c r="N9" t="str">
         <v>2027-07-31</v>
       </c>
-      <c r="M9" t="str">
-        <v>Không cải tạo lớn — chỉ mua TB mới nguyên căn.</v>
+      <c r="O9" t="str">
+        <v>Cải tạo nhẹ — chủ yếu mua TB mới nguyên căn.</v>
       </c>
     </row>
     <row r="10">
@@ -1394,24 +1450,30 @@
         <v>90</v>
       </c>
       <c r="G10">
+        <v>11.2</v>
+      </c>
+      <c r="H10">
+        <v>8</v>
+      </c>
+      <c r="I10">
         <v>3</v>
       </c>
-      <c r="H10">
+      <c r="J10">
         <v>4</v>
       </c>
-      <c r="I10" t="str">
+      <c r="K10" t="str">
         <v>Nguyễn Văn Hùng</v>
       </c>
-      <c r="J10">
+      <c r="L10">
         <v>240000000</v>
       </c>
-      <c r="K10" t="str">
+      <c r="M10" t="str">
         <v>2026-04-15</v>
       </c>
-      <c r="L10" t="str">
+      <c r="N10" t="str">
         <v>2029-04-14</v>
       </c>
-      <c r="M10" t="str">
+      <c r="O10" t="str">
         <v>Hà Nội — cải tạo tối thiểu 1 hạng mục.</v>
       </c>
     </row>
@@ -1435,24 +1497,30 @@
         <v>110</v>
       </c>
       <c r="G11">
+        <v>12.4</v>
+      </c>
+      <c r="H11">
+        <v>8.9</v>
+      </c>
+      <c r="I11">
         <v>2</v>
       </c>
-      <c r="H11">
+      <c r="J11">
         <v>3</v>
       </c>
-      <c r="I11" t="str">
+      <c r="K11" t="str">
         <v>Trịnh Quốc Anh</v>
       </c>
-      <c r="J11">
+      <c r="L11">
         <v>420000000</v>
       </c>
-      <c r="K11" t="str">
+      <c r="M11" t="str">
         <v>2026-10-01</v>
       </c>
-      <c r="L11" t="str">
+      <c r="N11" t="str">
         <v>2030-09-30</v>
       </c>
-      <c r="M11" t="str">
+      <c r="O11" t="str">
         <v>TB bàn giao nhiều trạng thái hỏng — không cải tạo.</v>
       </c>
     </row>
@@ -1476,24 +1544,30 @@
         <v>140</v>
       </c>
       <c r="G12">
+        <v>14</v>
+      </c>
+      <c r="H12">
+        <v>10</v>
+      </c>
+      <c r="I12">
         <v>2</v>
       </c>
-      <c r="H12">
+      <c r="J12">
         <v>6</v>
       </c>
-      <c r="I12" t="str">
+      <c r="K12" t="str">
         <v>Lý Thanh Tùng</v>
       </c>
-      <c r="J12">
+      <c r="L12">
         <v>360000000</v>
       </c>
-      <c r="K12" t="str">
+      <c r="M12" t="str">
         <v>2026-05-15</v>
       </c>
-      <c r="L12" t="str">
+      <c r="N12" t="str">
         <v>2030-05-14</v>
       </c>
-      <c r="M12" t="str">
+      <c r="O12" t="str">
         <v>Cải tạo kết cấu + nội thất nguyên căn.</v>
       </c>
     </row>
@@ -1517,24 +1591,30 @@
         <v>220</v>
       </c>
       <c r="G13">
+        <v>17.5</v>
+      </c>
+      <c r="H13">
+        <v>12.6</v>
+      </c>
+      <c r="I13">
         <v>4</v>
       </c>
-      <c r="H13">
+      <c r="J13">
         <v>14</v>
       </c>
-      <c r="I13" t="str">
+      <c r="K13" t="str">
         <v>Đỗ Thị Mai</v>
       </c>
-      <c r="J13">
+      <c r="L13">
         <v>520000000</v>
       </c>
-      <c r="K13" t="str">
+      <c r="M13" t="str">
         <v>2026-01-01</v>
       </c>
-      <c r="L13" t="str">
+      <c r="N13" t="str">
         <v>2030-12-31</v>
       </c>
-      <c r="M13" t="str">
+      <c r="O13" t="str">
         <v>Ký túc xá mini — 12 phòng khai thác.</v>
       </c>
     </row>
@@ -1558,24 +1638,30 @@
         <v>80</v>
       </c>
       <c r="G14">
+        <v>10.6</v>
+      </c>
+      <c r="H14">
+        <v>7.5</v>
+      </c>
+      <c r="I14">
         <v>2</v>
       </c>
-      <c r="H14">
+      <c r="J14">
         <v>3</v>
       </c>
-      <c r="I14" t="str">
+      <c r="K14" t="str">
         <v>Phan Minh Đức</v>
       </c>
-      <c r="J14">
+      <c r="L14">
         <v>200000000</v>
       </c>
-      <c r="K14" t="str">
+      <c r="M14" t="str">
         <v>2026-11-01</v>
       </c>
-      <c r="L14" t="str">
+      <c r="N14" t="str">
         <v>2028-10-31</v>
       </c>
-      <c r="M14" t="str">
+      <c r="O14" t="str">
         <v>Hà Nội — vào ở ngay, không cải tạo.</v>
       </c>
     </row>
@@ -1599,24 +1685,30 @@
         <v>250</v>
       </c>
       <c r="G15">
+        <v>18.7</v>
+      </c>
+      <c r="H15">
+        <v>13.4</v>
+      </c>
+      <c r="I15">
         <v>3</v>
       </c>
-      <c r="H15">
+      <c r="J15">
         <v>7</v>
       </c>
-      <c r="I15" t="str">
+      <c r="K15" t="str">
         <v>Vũ Thị Hồng</v>
       </c>
-      <c r="J15">
+      <c r="L15">
         <v>600000000</v>
       </c>
-      <c r="K15" t="str">
+      <c r="M15" t="str">
         <v>2026-03-15</v>
       </c>
-      <c r="L15" t="str">
+      <c r="N15" t="str">
         <v>2031-03-14</v>
       </c>
-      <c r="M15" t="str">
+      <c r="O15" t="str">
         <v>Biệt thự Hà Nội — cải tạo + mua TB cao cấp.</v>
       </c>
     </row>
@@ -1640,30 +1732,36 @@
         <v>100</v>
       </c>
       <c r="G16">
+        <v>11.8</v>
+      </c>
+      <c r="H16">
+        <v>8.5</v>
+      </c>
+      <c r="I16">
         <v>3</v>
       </c>
-      <c r="H16">
+      <c r="J16">
         <v>6</v>
       </c>
-      <c r="I16" t="str">
+      <c r="K16" t="str">
         <v>Trần Văn Phúc</v>
       </c>
-      <c r="J16">
+      <c r="L16">
         <v>270000000</v>
       </c>
-      <c r="K16" t="str">
+      <c r="M16" t="str">
         <v>2026-06-01</v>
       </c>
-      <c r="L16" t="str">
+      <c r="N16" t="str">
         <v>2028-05-31</v>
       </c>
-      <c r="M16" t="str">
+      <c r="O16" t="str">
         <v>Hà Nội — chia 5 phòng khai thác.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O16"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>